<commit_message>
precision recall and accuracy on the effect tab, plain code wording
</commit_message>
<xml_diff>
--- a/results/review/52_codes_no_icda8.xlsx
+++ b/results/review/52_codes_no_icda8.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">174 malignant neoplasm of breast</t>
   </si>
   <si>
-    <t xml:space="preserve">ICD-8 did not split breast cancer by sex. 174 malignant neoplasm of breast is the only breast rubric and it covers both</t>
+    <t xml:space="preserve">ICD-8 did not split breast cancer by sex. 174 malignant neoplasm of breast is the only breast code and it covers both</t>
   </si>
   <si>
     <t xml:space="preserve">176</t>
@@ -100,7 +100,7 @@
     <t xml:space="preserve">kaposis sarcoma</t>
   </si>
   <si>
-    <t xml:space="preserve">no Kaposi sarcoma rubric in ICD-8, it entered ICD-9-CM later</t>
+    <t xml:space="preserve">no Kaposi sarcoma code in ICD-8, it entered ICD-9-CM later</t>
   </si>
   <si>
     <t xml:space="preserve">179</t>
@@ -229,7 +229,7 @@
     <t xml:space="preserve">6 nervous system and sense organs</t>
   </si>
   <si>
-    <t xml:space="preserve">no sleep disorder rubric in ICD-8, organic sleep disorders entered ICD-9-CM in 2005</t>
+    <t xml:space="preserve">no sleep disorder code in ICD-8, organic sleep disorders entered ICD-9-CM in 2005</t>
   </si>
   <si>
     <t xml:space="preserve">330</t>
@@ -268,7 +268,7 @@
     <t xml:space="preserve">pain not elsewhere classified</t>
   </si>
   <si>
-    <t xml:space="preserve">no pain NEC rubric in ICD-8, it entered ICD-9-CM in 2006</t>
+    <t xml:space="preserve">no pain NEC code in ICD-8, it entered ICD-9-CM in 2006</t>
   </si>
   <si>
     <t xml:space="preserve">358</t>
@@ -313,7 +313,7 @@
     <t xml:space="preserve">8 respiratory system</t>
   </si>
   <si>
-    <t xml:space="preserve">extrinsic allergic alveolitis has no ICD-8 rubric</t>
+    <t xml:space="preserve">extrinsic allergic alveolitis has no ICD-8 code</t>
   </si>
   <si>
     <t xml:space="preserve">496</t>
@@ -361,7 +361,7 @@
     <t xml:space="preserve">563 chronic enteritis and ulcerative colitis</t>
   </si>
   <si>
-    <t xml:space="preserve">563 chronic enteritis and ulcerative colitis is the only chronic inflammatory bowel rubric in ICD-8, regional enteritis sits there</t>
+    <t xml:space="preserve">563 chronic enteritis and ulcerative colitis is the only chronic inflammatory bowel code in ICD-8, regional enteritis sits there</t>
   </si>
   <si>
     <t xml:space="preserve">557</t>
@@ -379,7 +379,7 @@
     <t xml:space="preserve">576 other diseases of gallbladder and biliary ducts</t>
   </si>
   <si>
-    <t xml:space="preserve">576 other diseases of gallbladder and biliary ducts is the same rubric under the same number</t>
+    <t xml:space="preserve">576 other diseases of gallbladder and biliary ducts is the same thing under the same number</t>
   </si>
   <si>
     <t xml:space="preserve">585</t>
@@ -466,7 +466,7 @@
     <t xml:space="preserve">746 congenital anomalies of heart</t>
   </si>
   <si>
-    <t xml:space="preserve">746 congenital anomalies of heart is the only heart rubric. Note ICD-8 745 is ear face and neck, the numbers do not line up between the two classifications</t>
+    <t xml:space="preserve">746 congenital anomalies of heart is the only heart code. Note ICD-8 745 is ear face and neck, the numbers do not line up between the two classifications</t>
   </si>
   <si>
     <t xml:space="preserve">codes with no ICDA-8 match</t>

</xml_diff>